<commit_message>
Add purchase and datasheet links for every BOM part; use 800 mA fuse
</commit_message>
<xml_diff>
--- a/docs/03-BOM/BOM_LiDAR_LK.xlsx
+++ b/docs/03-BOM/BOM_LiDAR_LK.xlsx
@@ -458,10 +458,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -634,7 +634,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>TO-220 Heatsink</t>
+          <t>Aavid 507002B00000G TO-220 Heatsink</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="E6" s="4">
         <f>C6*D6</f>
@@ -654,11 +654,19 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -691,12 +699,16 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>750 mA Slow-Blow Fuse, 5 × 20 mm</t>
+          <t>Littelfuse 0218.800MXP 800 mA Slow-Blow Fuse</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -708,7 +720,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E8" s="4">
         <f>C8*D8</f>
@@ -716,16 +728,24 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>BLX-A Fuse Holder, 5 × 20 mm</t>
+          <t>BLX-A Fuse Holder with Cover, 5 × 20 mm</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -753,12 +773,16 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>SS14 Schottky Diode</t>
+          <t>onsemi SS14 Schottky Diode</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -786,7 +810,11 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -811,11 +839,19 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -840,16 +876,24 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Shrouded IDC Header, 2 × 4</t>
+          <t>Würth 61200821621 Box Header, 2 × 4</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -869,16 +913,24 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Pin Header, 1 × 10</t>
+          <t>Würth 61301011121 Pin Header, 1 × 10</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -898,16 +950,24 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Pin Header, 1 × 2, with Jumper</t>
+          <t>Würth 61300211121 Pin Header, 1 × 2</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -919,7 +979,7 @@
         <v>5</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="E15" s="4">
         <f>C15*D15</f>
@@ -927,28 +987,36 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Green LED, 0805</t>
+          <t>Würth 60900213421 Jumper Shunt</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>D1, D4</t>
+          <t>JP1–JP5</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="E16" s="4">
         <f>C16*D16</f>
@@ -956,25 +1024,33 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Red LED, 0805</t>
+          <t>Würth 150080GS75000 Green LED, 0805</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D1, D4</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>0.25</v>
@@ -985,28 +1061,36 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Resistor, 1 kΩ, 0805</t>
+          <t>Würth 150080RS75000 Red LED, 0805</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>R1, R8</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="E18" s="4">
         <f>C18*D18</f>
@@ -1014,21 +1098,29 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Resistor, 330 Ω, 0805</t>
+          <t>Stackpole RMCF0805FT1K00 1 kΩ Resistor</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>R5, R6</t>
+          <t>R1, R8</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -1043,21 +1135,29 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Resistor, 10 kΩ, 0805</t>
+          <t>Stackpole RMCF0805FT330R 330 Ω Resistor</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>R4, R7</t>
+          <t>R5, R6</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -1072,25 +1172,33 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Resistor, 100 Ω, 0805</t>
+          <t>Stackpole RMCF0805FT10K0 10 kΩ Resistor</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R4, R7</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0.1</v>
@@ -1101,28 +1209,36 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 100 µF, 25 V, Electrolytic</t>
+          <t>Stackpole RMCF0805FT100R 100 Ω Resistor</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="E22" s="4">
         <f>C22*D22</f>
@@ -1130,28 +1246,36 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 22 µF, 16 V, Electrolytic</t>
+          <t>Panasonic EEU-FR1E101 100 µF 25 V Capacitor</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E23" s="4">
         <f>C23*D23</f>
@@ -1159,21 +1283,29 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 10 µF, 16 V, 0805</t>
+          <t>Panasonic EEU-FR1C220 22 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -1188,28 +1320,36 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 1 µF, 16 V, 0805</t>
+          <t>Samsung CL21A106KOQNNNE 10 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E25" s="4">
         <f>C25*D25</f>
@@ -1217,21 +1357,29 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 0.47 µF, 50 V, 0805</t>
+          <t>Samsung CL21B105KOFNNNE 1 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -1246,25 +1394,33 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Capacitor, 0.1 µF, 50 V, 0805</t>
+          <t>Samsung CL21B474KBFNNNE 0.47 µF 50 V Capacitor</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>C4, C5, C6, C8</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D27" s="4" t="n">
         <v>0.1</v>
@@ -1275,28 +1431,73 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Generic</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Samsung CL21B104KBCNNNC 0.1 µF 50 V Capacitor</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>C4, C5, C6, C8</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="4">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>DigiKey</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Total estimated cost</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="7">
-        <f>SUM(E3:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="7">
+        <f>SUM(E3:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1309,9 +1510,52 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use Amazon kits in BOM where practical; keep 750 mA fuse
</commit_message>
<xml_diff>
--- a/docs/03-BOM/BOM_LiDAR_LK.xlsx
+++ b/docs/03-BOM/BOM_LiDAR_LK.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>TI LM2940CT-5.0 5 V Regulator</t>
+          <t>LM2940CT-5.0 5 V Regulator (Chanzon 10-pack)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>1.94</v>
+        <v>7.99</v>
       </c>
       <c r="E5" s="4">
         <f>C5*D5</f>
@@ -617,7 +617,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Aavid 507002B00000G TO-220 Heatsink</t>
+          <t>TO-220 Heatsink (Heyous 30-pack)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.7</v>
+        <v>7.99</v>
       </c>
       <c r="E6" s="4">
         <f>C6*D6</f>
@@ -654,7 +654,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -708,7 +708,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Littelfuse 0218.800MXP 800 mA Slow-Blow Fuse</t>
+          <t>T750mA 250 V Slow-Blow Fuse, 5 × 20 mm (20-pack)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.4</v>
+        <v>7.99</v>
       </c>
       <c r="E8" s="4">
         <f>C8*D8</f>
@@ -728,7 +728,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -930,7 +930,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Würth 61301011121 Pin Header, 1 × 10</t>
+          <t>2.54 mm Header Kit, 1 × 10 (QSYZAIL 122-pc kit)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -939,10 +939,10 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.5</v>
+        <v>9.99</v>
       </c>
       <c r="E14" s="4">
         <f>C14*D14</f>
@@ -950,7 +950,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1115,19 +1115,19 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Stackpole RMCF0805FT1K00 1 kΩ Resistor</t>
+          <t>0805 Resistors: 1 kΩ, 330 Ω, 10 kΩ, 100 Ω (EGSCST 0805 kit)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>R1, R8</t>
+          <t>R1, R2, R4–R8</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.1</v>
+        <v>36.9</v>
       </c>
       <c r="E19" s="4">
         <f>C19*D19</f>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1152,19 +1152,19 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Stackpole RMCF0805FT330R 330 Ω Resistor</t>
+          <t>Electrolytic Capacitors: 100 µF 25 V, 22 µF 16 V (Tnisesm kit)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>R5, R6</t>
+          <t>C1, C3</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0.1</v>
+        <v>8.99</v>
       </c>
       <c r="E20" s="4">
         <f>C20*D20</f>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1189,19 +1189,19 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Stackpole RMCF0805FT10K0 10 kΩ Resistor</t>
+          <t>Samsung CL21A106KOQNNNE 10 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>R4, R7</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E21" s="4">
         <f>C21*D21</f>
@@ -1226,12 +1226,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Stackpole RMCF0805FT100R 100 Ω Resistor</t>
+          <t>Samsung CL21B105KOFNNNE 1 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -1263,19 +1263,19 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Panasonic EEU-FR1E101 100 µF 25 V Capacitor</t>
+          <t>Samsung CL21B474KBFNNNE 0.47 µF 50 V Capacitor</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E23" s="4">
         <f>C23*D23</f>
@@ -1300,19 +1300,19 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Panasonic EEU-FR1C220 22 µF 16 V Capacitor</t>
+          <t>Samsung CL21B104KBCNNNC 0.1 µF 50 V Capacitor</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4, C5, C6, C8</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="E24" s="4">
         <f>C24*D24</f>
@@ -1335,169 +1335,21 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Samsung CL21A106KOQNNNE 10 µF 16 V Capacitor</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>C7</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E25" s="4">
-        <f>C25*D25</f>
-        <v/>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>View Product</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Samsung CL21B105KOFNNNE 1 µF 16 V Capacitor</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>C9</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E26" s="4">
-        <f>C26*D26</f>
-        <v/>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>View Product</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Samsung CL21B474KBFNNNE 0.47 µF 50 V Capacitor</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E27" s="4">
-        <f>C27*D27</f>
-        <v/>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>View Product</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Samsung CL21B104KBCNNNC 0.1 µF 50 V Capacitor</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>C4, C5, C6, C8</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E28" s="4">
-        <f>C28*D28</f>
-        <v/>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>View Product</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Total estimated cost</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr"/>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="7">
-        <f>SUM(E3:E28)</f>
-        <v/>
-      </c>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="7">
+        <f>SUM(E3:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1548,14 +1400,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Order board parts from DigiKey; 0805 book supplies resistors, capacitors, and LEDs
</commit_message>
<xml_diff>
--- a/docs/03-BOM/BOM_LiDAR_LK.xlsx
+++ b/docs/03-BOM/BOM_LiDAR_LK.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>LM2940CT-5.0 5 V Regulator (Chanzon 10-pack)</t>
+          <t>TI LM2940CT-5.0 5 V Regulator</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>7.99</v>
+        <v>1.94</v>
       </c>
       <c r="E5" s="4">
         <f>C5*D5</f>
@@ -617,7 +617,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>TO-220 Heatsink (Heyous 30-pack)</t>
+          <t>Aavid 507002B00000G TO-220 Heatsink</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>7.99</v>
+        <v>0.7</v>
       </c>
       <c r="E6" s="4">
         <f>C6*D6</f>
@@ -654,7 +654,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -708,7 +708,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T750mA 250 V Slow-Blow Fuse, 5 × 20 mm (20-pack)</t>
+          <t>Eaton GMC-750-R 750 mA Slow-Blow Fuse, 5 × 20 mm</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>7.99</v>
+        <v>0.7</v>
       </c>
       <c r="E8" s="4">
         <f>C8*D8</f>
@@ -728,7 +728,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -930,7 +930,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2.54 mm Header Kit, 1 × 10 (QSYZAIL 122-pc kit)</t>
+          <t>Würth 61301011121 Pin Header, 1 × 10</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -939,10 +939,10 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>9.99</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="4">
         <f>C14*D14</f>
@@ -950,7 +950,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1041,19 +1041,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Würth 150080GS75000 Green LED, 0805</t>
+          <t>Panasonic EEU-FR1E101 100 µF 25 V Capacitor</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>D1, D4</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="E17" s="4">
         <f>C17*D17</f>
@@ -1078,12 +1078,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Würth 150080RS75000 Red LED, 0805</t>
+          <t>Panasonic EEU-FR1C220 22 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -1115,12 +1115,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>0805 Resistors: 1 kΩ, 330 Ω, 10 kΩ, 100 Ω (EGSCST 0805 kit)</t>
+          <t>EGSCST 0805 SMD Component Book (5600 pcs)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>R1, R2, R4–R8</t>
+          <t>Parts below</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -1143,28 +1143,24 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
+      <c r="H19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Electrolytic Capacitors: 100 µF 25 V, 22 µF 16 V (Tnisesm kit)</t>
+          <t>0805 Resistors: 1 kΩ, 330 Ω, 10 kΩ, 100 Ω</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>C1, C3</t>
+          <t>R1, R2, R4–R8</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>8.99</v>
+        <v>0</v>
       </c>
       <c r="E20" s="4">
         <f>C20*D20</f>
@@ -1172,7 +1168,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>In book</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1189,7 +1185,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL21A106KOQNNNE 10 µF 16 V Capacitor</t>
+          <t>0805 Capacitor, 10 µF</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1201,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E21" s="4">
         <f>C21*D21</f>
@@ -1209,7 +1205,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>In book</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1226,7 +1222,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL21B105KOFNNNE 1 µF 16 V Capacitor</t>
+          <t>0805 Capacitor, 1 µF</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1238,7 +1234,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="4">
         <f>C22*D22</f>
@@ -1246,7 +1242,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>In book</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1263,7 +1259,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL21B474KBFNNNE 0.47 µF 50 V Capacitor</t>
+          <t>0805 Capacitor, 0.47 µF</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1275,7 +1271,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="4">
         <f>C23*D23</f>
@@ -1283,7 +1279,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>In book</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
@@ -1300,7 +1296,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Samsung CL21B104KBCNNNC 0.1 µF 50 V Capacitor</t>
+          <t>0805 Capacitor, 0.1 µF</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1312,7 +1308,7 @@
         <v>4</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E24" s="4">
         <f>C24*D24</f>
@@ -1320,7 +1316,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>In book</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1335,21 +1331,58 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>0805 LEDs, Green and Red</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>D1, D3, D4</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>In book</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Total estimated cost</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr"/>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="7">
-        <f>SUM(E3:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="7">
+        <f>SUM(E3:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1389,17 +1422,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark fuse holder as already on hand
</commit_message>
<xml_diff>
--- a/docs/03-BOM/BOM_LiDAR_LK.xlsx
+++ b/docs/03-BOM/BOM_LiDAR_LK.xlsx
@@ -745,7 +745,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>BLX-A Fuse Holder with Cover, 5 × 20 mm</t>
+          <t>BLX-A Fuse Holder with Cover, 5 × 20 mm (already have, from kit)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -757,7 +757,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4">
         <f>C9*D9</f>
@@ -765,7 +765,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Tayda</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Mark team ribbon cable, headers, and jumpers as already on hand
</commit_message>
<xml_diff>
--- a/docs/03-BOM/BOM_LiDAR_LK.xlsx
+++ b/docs/03-BOM/BOM_LiDAR_LK.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -893,7 +893,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Würth 61200821621 Box Header, 2 × 4</t>
+          <t>Würth 61200821621 Box Header, 2 × 4 (already have, from kit)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -905,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E13" s="4">
         <f>C13*D13</f>
@@ -913,7 +913,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -930,19 +930,19 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Würth 61301011121 Pin Header, 1 × 10</t>
+          <t>8-Wire Ribbon Cable with 2 × 4 IDC Connectors (already have, from kit)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>J4, J5</t>
+          <t>To J3</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E14" s="4">
         <f>C14*D14</f>
@@ -950,7 +950,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -958,28 +958,24 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Würth 61300211121 Pin Header, 1 × 2</t>
+          <t>Würth 61301011121 Pin Header, 1 × 10 (already have, from kit)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>JP1–JP5</t>
+          <t>J4, J5</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E15" s="4">
         <f>C15*D15</f>
@@ -987,7 +983,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1004,7 +1000,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Würth 60900213421 Jumper Shunt</t>
+          <t>Würth 61300211121 Pin Header, 1 × 2 (already have, from kit)</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1016,7 +1012,7 @@
         <v>5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E16" s="4">
         <f>C16*D16</f>
@@ -1024,7 +1020,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1041,19 +1037,19 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Panasonic EEU-FR1E101 100 µF 25 V Capacitor</t>
+          <t>Würth 60900213421 Jumper Shunt (already have, from kit)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>JP1–JP5</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="E17" s="4">
         <f>C17*D17</f>
@@ -1061,7 +1057,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Have</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1078,19 +1074,19 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Panasonic EEU-FR1C220 22 µF 16 V Capacitor</t>
+          <t>Panasonic EEU-FR1E101 100 µF 25 V Capacitor</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="E18" s="4">
         <f>C18*D18</f>
@@ -1115,19 +1111,19 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>EGSCST 0805 SMD Component Book (5600 pcs)</t>
+          <t>Panasonic EEU-FR1C220 22 µF 16 V Capacitor</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Parts below</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>36.9</v>
+        <v>0.25</v>
       </c>
       <c r="E19" s="4">
         <f>C19*D19</f>
@@ -1135,7 +1131,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1143,24 +1139,28 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>0805 Resistors: 1 kΩ, 330 Ω, 10 kΩ, 100 Ω</t>
+          <t>EGSCST 0805 SMD Component Book (5600 pcs)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>R1, R2, R4–R8</t>
+          <t>Parts below</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0</v>
+        <v>36.9</v>
       </c>
       <c r="E20" s="4">
         <f>C20*D20</f>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>In book</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1176,25 +1176,21 @@
           <t>View Product</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>View Datasheet</t>
-        </is>
-      </c>
+      <c r="H20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>0805 Capacitor, 10 µF</t>
+          <t>0805 Resistors: 1 kΩ, 330 Ω, 10 kΩ, 100 Ω</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>R1, R2, R4–R8</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -1222,12 +1218,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>0805 Capacitor, 1 µF</t>
+          <t>0805 Capacitor, 10 µF</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -1259,12 +1255,12 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>0805 Capacitor, 0.47 µF</t>
+          <t>0805 Capacitor, 1 µF</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C9</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -1296,16 +1292,16 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>0805 Capacitor, 0.1 µF</t>
+          <t>0805 Capacitor, 0.47 µF</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>C4, C5, C6, C8</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>0</v>
@@ -1333,16 +1329,16 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>0805 LEDs, Green and Red</t>
+          <t>0805 Capacitor, 0.1 µF</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>D1, D3, D4</t>
+          <t>C4, C5, C6, C8</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>0</v>
@@ -1368,21 +1364,58 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>0805 LEDs, Green and Red</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>D1, D3, D4</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>In book</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>View Product</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>View Datasheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Total estimated cost</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="7">
-        <f>SUM(E3:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="7">
+        <f>SUM(E3:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1412,28 +1445,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>